<commit_message>
Netflix - huge expectations priced in
</commit_message>
<xml_diff>
--- a/Visa.xlsx
+++ b/Visa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Github Financial Models\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59407837-3717-44E4-A208-0D8786695D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB41A267-D5BA-4750-8158-DA96BF894E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" activeTab="1" xr2:uid="{60472900-A3C3-4A5B-9BFF-D960E46989EA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{60472900-A3C3-4A5B-9BFF-D960E46989EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Financials" sheetId="1" r:id="rId1"/>
@@ -542,7 +542,7 @@
   <numFmts count="3">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -592,21 +592,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -973,7 +970,7 @@
       <c r="L1" t="s">
         <v>16</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="9" t="s">
         <v>13</v>
       </c>
       <c r="N1" s="2" t="s">
@@ -1077,7 +1074,7 @@
       <c r="L2" s="4">
         <v>8123</v>
       </c>
-      <c r="M2" s="12">
+      <c r="M2" s="10">
         <f xml:space="preserve"> I2*1.1</f>
         <v>8565.7000000000007</v>
       </c>
@@ -1093,75 +1090,75 @@
         <f>SUM(J2:M2)</f>
         <v>32609.7</v>
       </c>
-      <c r="R2" s="12">
+      <c r="R2" s="10">
         <f xml:space="preserve"> Q2*1.15</f>
         <v>37501.154999999999</v>
       </c>
-      <c r="S2" s="12">
+      <c r="S2" s="10">
         <f xml:space="preserve"> R2*1.15</f>
         <v>43126.328249999999</v>
       </c>
-      <c r="T2" s="12">
+      <c r="T2" s="10">
         <f xml:space="preserve"> S2*1.15</f>
         <v>49595.277487499996</v>
       </c>
-      <c r="U2" s="12">
+      <c r="U2" s="10">
         <f xml:space="preserve"> T2*1.15</f>
         <v>57034.569110624994</v>
       </c>
-      <c r="V2" s="12">
+      <c r="V2" s="10">
         <f xml:space="preserve"> U2*1.15</f>
         <v>65589.754477218739</v>
       </c>
-      <c r="W2" s="12">
+      <c r="W2" s="10">
         <f xml:space="preserve"> V2*1.15</f>
         <v>75428.217648801539</v>
       </c>
-      <c r="X2" s="12">
+      <c r="X2" s="10">
         <f xml:space="preserve"> W2*1.15</f>
         <v>86742.450296121766</v>
       </c>
-      <c r="Y2" s="12">
+      <c r="Y2" s="10">
         <f xml:space="preserve"> X2*1.15</f>
         <v>99753.817840540025</v>
       </c>
-      <c r="Z2" s="12">
+      <c r="Z2" s="10">
         <f xml:space="preserve"> Y2*1.15</f>
         <v>114716.89051662102</v>
       </c>
-      <c r="AA2" s="12">
+      <c r="AA2" s="10">
         <f xml:space="preserve"> Z2*1.15</f>
         <v>131924.42409411416</v>
       </c>
-      <c r="AB2" s="12">
+      <c r="AB2" s="10">
         <f xml:space="preserve"> AA2*1.15</f>
         <v>151713.08770823127</v>
       </c>
-      <c r="AC2" s="12">
+      <c r="AC2" s="10">
         <f xml:space="preserve"> AB2*1.15</f>
         <v>174470.05086446594</v>
       </c>
-      <c r="AD2" s="12">
+      <c r="AD2" s="10">
         <f xml:space="preserve"> AC2*1.15</f>
         <v>200640.55849413582</v>
       </c>
-      <c r="AE2" s="12">
+      <c r="AE2" s="10">
         <f xml:space="preserve"> AD2*1.15</f>
         <v>230736.64226825617</v>
       </c>
-      <c r="AF2" s="12">
+      <c r="AF2" s="10">
         <f xml:space="preserve"> AE2*1.15</f>
         <v>265347.1386084946</v>
       </c>
-      <c r="AG2" s="12">
+      <c r="AG2" s="10">
         <f xml:space="preserve"> AF2*1.15</f>
         <v>305149.20939976879</v>
       </c>
-      <c r="AH2" s="12">
+      <c r="AH2" s="10">
         <f xml:space="preserve"> AG2*1.15</f>
         <v>350921.59080973407</v>
       </c>
-      <c r="XFD2" s="12"/>
+      <c r="XFD2" s="10"/>
     </row>
     <row r="3" spans="1:34 16384:16384" x14ac:dyDescent="0.2">
       <c r="B3" s="3"/>
@@ -1232,15 +1229,15 @@
       <c r="M5" s="7">
         <v>1400</v>
       </c>
-      <c r="O5" s="13">
-        <f>SUM(B5:E5)</f>
+      <c r="O5" s="5">
+        <f t="shared" ref="O5:O13" si="0">SUM(B5:E5)</f>
         <v>4240</v>
       </c>
       <c r="P5" s="5">
         <f xml:space="preserve"> SUM(F5:I5)</f>
         <v>4990</v>
       </c>
-      <c r="Q5" s="13">
+      <c r="Q5" s="5">
         <f>SUM(J5:M5)</f>
         <v>5733</v>
       </c>
@@ -1285,16 +1282,16 @@
       <c r="M6" s="3">
         <v>300</v>
       </c>
-      <c r="O6" s="13">
-        <f>SUM(B6:E6)</f>
+      <c r="O6" s="5">
+        <f t="shared" si="0"/>
         <v>1136</v>
       </c>
       <c r="P6" s="5">
-        <f t="shared" ref="P6:P13" si="0" xml:space="preserve"> SUM(F6:I6)</f>
+        <f t="shared" ref="P6:P13" si="1" xml:space="preserve"> SUM(F6:I6)</f>
         <v>1336</v>
       </c>
-      <c r="Q6" s="13">
-        <f t="shared" ref="Q6:Q21" si="1">SUM(J6:M6)</f>
+      <c r="Q6" s="5">
+        <f t="shared" ref="Q6:Q21" si="2">SUM(J6:M6)</f>
         <v>1238</v>
       </c>
     </row>
@@ -1338,16 +1335,16 @@
       <c r="M7" s="3">
         <v>182</v>
       </c>
-      <c r="O7" s="13">
-        <f>SUM(B7:E7)</f>
+      <c r="O7" s="5">
+        <f t="shared" si="0"/>
         <v>730</v>
       </c>
       <c r="P7" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>743</v>
       </c>
-      <c r="Q7" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q7" s="5">
+        <f t="shared" si="2"/>
         <v>721</v>
       </c>
     </row>
@@ -1391,16 +1388,16 @@
       <c r="M8" s="3">
         <v>133</v>
       </c>
-      <c r="O8" s="13">
-        <f>SUM(B8:E8)</f>
+      <c r="O8" s="5">
+        <f t="shared" si="0"/>
         <v>403</v>
       </c>
       <c r="P8" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>505</v>
       </c>
-      <c r="Q8" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q8" s="5">
+        <f t="shared" si="2"/>
         <v>505</v>
       </c>
     </row>
@@ -1444,16 +1441,16 @@
       <c r="M9" s="3">
         <v>235</v>
       </c>
-      <c r="O9" s="13">
-        <f>SUM(B9:E9)</f>
+      <c r="O9" s="5">
+        <f t="shared" si="0"/>
         <v>804</v>
       </c>
       <c r="P9" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>861</v>
       </c>
-      <c r="Q9" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q9" s="5">
+        <f t="shared" si="2"/>
         <v>931</v>
       </c>
     </row>
@@ -1497,16 +1494,16 @@
       <c r="M10" s="3">
         <v>314</v>
       </c>
-      <c r="O10" s="13">
-        <f>SUM(B10:E10)</f>
+      <c r="O10" s="5">
+        <f t="shared" si="0"/>
         <v>985</v>
       </c>
       <c r="P10" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1194</v>
       </c>
-      <c r="Q10" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q10" s="5">
+        <f t="shared" si="2"/>
         <v>1232</v>
       </c>
     </row>
@@ -1550,16 +1547,16 @@
       <c r="M11" s="3">
         <v>457</v>
       </c>
-      <c r="O11" s="13">
-        <f>SUM(B11:E11)</f>
+      <c r="O11" s="5">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="P11" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>868</v>
       </c>
-      <c r="Q11" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q11" s="5">
+        <f t="shared" si="2"/>
         <v>1255</v>
       </c>
     </row>
@@ -1568,63 +1565,63 @@
         <v>24</v>
       </c>
       <c r="B12" s="4">
-        <f>SUM(B5:B11)</f>
+        <f t="shared" ref="B12:M12" si="3">SUM(B5:B11)</f>
         <v>1843</v>
       </c>
       <c r="C12" s="4">
-        <f>SUM(C5:C11)</f>
+        <f t="shared" si="3"/>
         <v>2148</v>
       </c>
       <c r="D12" s="4">
-        <f>SUM(D5:D11)</f>
+        <f t="shared" si="3"/>
         <v>2066</v>
       </c>
       <c r="E12" s="4">
-        <f>SUM(E5:E11)</f>
+        <f t="shared" si="3"/>
         <v>2244</v>
       </c>
       <c r="F12" s="4">
-        <f>SUM(F5:F11)</f>
+        <f t="shared" si="3"/>
         <v>2283</v>
       </c>
       <c r="G12" s="4">
-        <f>SUM(G5:G11)</f>
+        <f t="shared" si="3"/>
         <v>2387</v>
       </c>
       <c r="H12" s="4">
-        <f>SUM(H5:H11)</f>
+        <f t="shared" si="3"/>
         <v>3127</v>
       </c>
       <c r="I12" s="4">
-        <f>SUM(I5:I11)</f>
+        <f t="shared" si="3"/>
         <v>2700</v>
       </c>
       <c r="J12" s="4">
-        <f>SUM(J5:J11)</f>
+        <f t="shared" si="3"/>
         <v>2846</v>
       </c>
       <c r="K12" s="4">
-        <f>SUM(K5:K11)</f>
+        <f t="shared" si="3"/>
         <v>2649</v>
       </c>
       <c r="L12" s="4">
-        <f>SUM(L5:L11)</f>
+        <f t="shared" si="3"/>
         <v>3099</v>
       </c>
       <c r="M12" s="4">
-        <f>SUM(M5:M11)</f>
+        <f t="shared" si="3"/>
         <v>3021</v>
       </c>
       <c r="O12" s="6">
-        <f>SUM(B12:E12)</f>
+        <f t="shared" si="0"/>
         <v>8301</v>
       </c>
       <c r="P12" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10497</v>
       </c>
       <c r="Q12" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11615</v>
       </c>
     </row>
@@ -1633,69 +1630,69 @@
         <v>36</v>
       </c>
       <c r="B13" s="4">
-        <f xml:space="preserve"> B2 -B12</f>
+        <f t="shared" ref="B13:M13" si="4" xml:space="preserve"> B2 -B12</f>
         <v>3844</v>
       </c>
       <c r="C13" s="4">
-        <f xml:space="preserve"> C2 -C12</f>
+        <f t="shared" si="4"/>
         <v>3581</v>
       </c>
       <c r="D13" s="4">
-        <f xml:space="preserve"> D2 -D12</f>
+        <f t="shared" si="4"/>
         <v>4064</v>
       </c>
       <c r="E13" s="4">
-        <f xml:space="preserve"> E2 -E12</f>
+        <f t="shared" si="4"/>
         <v>4315</v>
       </c>
       <c r="F13" s="4">
-        <f xml:space="preserve"> F2 -F12</f>
+        <f t="shared" si="4"/>
         <v>4776</v>
       </c>
       <c r="G13" s="4">
-        <f xml:space="preserve"> G2 -G12</f>
+        <f t="shared" si="4"/>
         <v>4802</v>
       </c>
       <c r="H13" s="4">
-        <f xml:space="preserve"> H2 -H12</f>
+        <f t="shared" si="4"/>
         <v>4148</v>
       </c>
       <c r="I13" s="4">
-        <f xml:space="preserve"> I2 -I12</f>
+        <f t="shared" si="4"/>
         <v>5087</v>
       </c>
       <c r="J13" s="4">
-        <f xml:space="preserve"> J2 -J12</f>
+        <f t="shared" si="4"/>
         <v>5090</v>
       </c>
       <c r="K13" s="4">
-        <f xml:space="preserve"> K2 -K12</f>
+        <f t="shared" si="4"/>
         <v>5336</v>
       </c>
       <c r="L13" s="4">
-        <f xml:space="preserve"> L2 -L12</f>
+        <f t="shared" si="4"/>
         <v>5024</v>
       </c>
       <c r="M13" s="4">
-        <f xml:space="preserve"> M2 -M12</f>
+        <f t="shared" si="4"/>
         <v>5544.7000000000007</v>
       </c>
       <c r="O13" s="6">
-        <f>SUM(B13:E13)</f>
+        <f t="shared" si="0"/>
         <v>15804</v>
       </c>
       <c r="P13" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18813</v>
       </c>
       <c r="Q13" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20994.7</v>
       </c>
     </row>
     <row r="14" spans="1:34 16384:16384" x14ac:dyDescent="0.2">
-      <c r="Q14" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q14" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1703,8 +1700,8 @@
       <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Q15" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q15" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1748,16 +1745,16 @@
       <c r="M16">
         <v>-182</v>
       </c>
-      <c r="O16" s="13">
-        <f>SUM(B16:E16)</f>
+      <c r="O16" s="5">
+        <f t="shared" ref="O16:O21" si="5">SUM(B16:E16)</f>
         <v>-513</v>
       </c>
       <c r="P16" s="5">
-        <f t="shared" ref="P16:P21" si="2" xml:space="preserve"> SUM(F16:I16)</f>
+        <f t="shared" ref="P16:P21" si="6" xml:space="preserve"> SUM(F16:I16)</f>
         <v>-538</v>
       </c>
-      <c r="Q16" s="13">
-        <f t="shared" si="1"/>
+      <c r="Q16" s="5">
+        <f t="shared" si="2"/>
         <v>-643</v>
       </c>
     </row>
@@ -1801,16 +1798,16 @@
       <c r="M17">
         <v>304</v>
       </c>
-      <c r="O17" s="13">
-        <f>SUM(B17:E17)</f>
+      <c r="O17" s="5">
+        <f t="shared" si="5"/>
         <v>772</v>
       </c>
       <c r="P17" s="5">
+        <f t="shared" si="6"/>
+        <v>-139</v>
+      </c>
+      <c r="Q17" s="5">
         <f t="shared" si="2"/>
-        <v>-139</v>
-      </c>
-      <c r="Q17" s="13">
-        <f t="shared" si="1"/>
         <v>716</v>
       </c>
     </row>
@@ -1819,63 +1816,63 @@
         <v>40</v>
       </c>
       <c r="B18">
-        <f xml:space="preserve"> SUM(B16:B17)</f>
+        <f t="shared" ref="B18:M18" si="7" xml:space="preserve"> SUM(B16:B17)</f>
         <v>-96</v>
       </c>
       <c r="C18">
-        <f xml:space="preserve"> SUM(C16:C17)</f>
+        <f t="shared" si="7"/>
         <v>47</v>
       </c>
       <c r="D18">
-        <f xml:space="preserve"> SUM(D16:D17)</f>
+        <f t="shared" si="7"/>
         <v>325</v>
       </c>
       <c r="E18">
-        <f xml:space="preserve"> SUM(E16:E17)</f>
+        <f t="shared" si="7"/>
         <v>-17</v>
       </c>
       <c r="F18">
-        <f xml:space="preserve"> SUM(F16:F17)</f>
+        <f t="shared" si="7"/>
         <v>121</v>
       </c>
       <c r="G18">
-        <f xml:space="preserve"> SUM(G16:G17)</f>
+        <f t="shared" si="7"/>
         <v>-260</v>
       </c>
       <c r="H18">
-        <f xml:space="preserve"> SUM(H16:H17)</f>
+        <f t="shared" si="7"/>
         <v>-319</v>
       </c>
       <c r="I18">
-        <f xml:space="preserve"> SUM(I16:I17)</f>
+        <f t="shared" si="7"/>
         <v>-219</v>
       </c>
       <c r="J18">
-        <f xml:space="preserve"> SUM(J16:J17)</f>
+        <f t="shared" si="7"/>
         <v>-113</v>
       </c>
       <c r="K18">
-        <f xml:space="preserve"> SUM(K16:K17)</f>
+        <f t="shared" si="7"/>
         <v>-58</v>
       </c>
       <c r="L18">
-        <f xml:space="preserve"> SUM(L16:L17)</f>
+        <f t="shared" si="7"/>
         <v>122</v>
       </c>
       <c r="M18">
-        <f xml:space="preserve"> SUM(M16:M17)</f>
+        <f t="shared" si="7"/>
         <v>122</v>
       </c>
-      <c r="O18" s="13">
-        <f>SUM(B18:E18)</f>
+      <c r="O18" s="5">
+        <f t="shared" si="5"/>
         <v>259</v>
       </c>
       <c r="P18" s="5">
+        <f t="shared" si="6"/>
+        <v>-677</v>
+      </c>
+      <c r="Q18" s="5">
         <f t="shared" si="2"/>
-        <v>-677</v>
-      </c>
-      <c r="Q18" s="13">
-        <f t="shared" si="1"/>
         <v>73</v>
       </c>
     </row>
@@ -1884,63 +1881,63 @@
         <v>41</v>
       </c>
       <c r="B19" s="6">
-        <f xml:space="preserve"> B13 + B18</f>
+        <f t="shared" ref="B19:M19" si="8" xml:space="preserve"> B13 + B18</f>
         <v>3748</v>
       </c>
       <c r="C19" s="6">
-        <f xml:space="preserve"> C13 + C18</f>
+        <f t="shared" si="8"/>
         <v>3628</v>
       </c>
       <c r="D19" s="6">
-        <f xml:space="preserve"> D13 + D18</f>
+        <f t="shared" si="8"/>
         <v>4389</v>
       </c>
       <c r="E19" s="6">
-        <f xml:space="preserve"> E13 + E18</f>
+        <f t="shared" si="8"/>
         <v>4298</v>
       </c>
       <c r="F19" s="6">
-        <f xml:space="preserve"> F13 + F18</f>
+        <f t="shared" si="8"/>
         <v>4897</v>
       </c>
       <c r="G19" s="6">
-        <f xml:space="preserve"> G13 + G18</f>
+        <f t="shared" si="8"/>
         <v>4542</v>
       </c>
       <c r="H19" s="6">
-        <f xml:space="preserve"> H13 + H18</f>
+        <f t="shared" si="8"/>
         <v>3829</v>
       </c>
       <c r="I19" s="6">
-        <f xml:space="preserve"> I13 + I18</f>
+        <f t="shared" si="8"/>
         <v>4868</v>
       </c>
       <c r="J19" s="6">
-        <f xml:space="preserve"> J13 + J18</f>
+        <f t="shared" si="8"/>
         <v>4977</v>
       </c>
       <c r="K19" s="6">
-        <f xml:space="preserve"> K13 + K18</f>
+        <f t="shared" si="8"/>
         <v>5278</v>
       </c>
       <c r="L19" s="6">
-        <f xml:space="preserve"> L13 + L18</f>
+        <f t="shared" si="8"/>
         <v>5146</v>
       </c>
       <c r="M19" s="6">
-        <f xml:space="preserve"> M13 + M18</f>
+        <f t="shared" si="8"/>
         <v>5666.7000000000007</v>
       </c>
       <c r="O19" s="6">
-        <f>SUM(B19:E19)</f>
+        <f t="shared" si="5"/>
         <v>16063</v>
       </c>
       <c r="P19" s="6">
+        <f t="shared" si="6"/>
+        <v>18136</v>
+      </c>
+      <c r="Q19" s="6">
         <f t="shared" si="2"/>
-        <v>18136</v>
-      </c>
-      <c r="Q19" s="6">
-        <f t="shared" si="1"/>
         <v>21067.7</v>
       </c>
     </row>
@@ -1984,16 +1981,16 @@
       <c r="M20">
         <v>1100</v>
       </c>
-      <c r="O20" s="13">
-        <f>SUM(B20:E20)</f>
+      <c r="O20" s="5">
+        <f t="shared" si="5"/>
         <v>3752</v>
       </c>
       <c r="P20" s="5">
+        <f t="shared" si="6"/>
+        <v>3179</v>
+      </c>
+      <c r="Q20" s="5">
         <f t="shared" si="2"/>
-        <v>3179</v>
-      </c>
-      <c r="Q20" s="13">
-        <f t="shared" si="1"/>
         <v>3909</v>
       </c>
     </row>
@@ -2002,196 +1999,196 @@
         <v>27</v>
       </c>
       <c r="B21" s="6">
-        <f>B19 - B20</f>
+        <f t="shared" ref="B21:M21" si="9">B19 - B20</f>
         <v>3126</v>
       </c>
       <c r="C21" s="6">
-        <f>C19 - C20</f>
+        <f t="shared" si="9"/>
         <v>3026</v>
       </c>
       <c r="D21" s="6">
-        <f>D19 - D20</f>
+        <f t="shared" si="9"/>
         <v>2575</v>
       </c>
       <c r="E21" s="6">
-        <f>E19 - E20</f>
+        <f t="shared" si="9"/>
         <v>3584</v>
       </c>
       <c r="F21" s="6">
-        <f>F19 - F20</f>
+        <f t="shared" si="9"/>
         <v>3959</v>
       </c>
       <c r="G21" s="6">
-        <f>G19 - G20</f>
+        <f t="shared" si="9"/>
         <v>3647</v>
       </c>
       <c r="H21" s="6">
-        <f>H19 - H20</f>
+        <f t="shared" si="9"/>
         <v>3411</v>
       </c>
       <c r="I21" s="6">
-        <f>I19 - I20</f>
+        <f t="shared" si="9"/>
         <v>3940</v>
       </c>
       <c r="J21" s="6">
-        <f>J19 - J20</f>
+        <f t="shared" si="9"/>
         <v>4179</v>
       </c>
       <c r="K21" s="6">
-        <f>K19 - K20</f>
+        <f t="shared" si="9"/>
         <v>4257</v>
       </c>
       <c r="L21" s="6">
-        <f>L19 - L20</f>
+        <f t="shared" si="9"/>
         <v>4156</v>
       </c>
       <c r="M21" s="6">
-        <f>M19 - M20</f>
+        <f t="shared" si="9"/>
         <v>4566.7000000000007</v>
       </c>
       <c r="O21" s="6">
-        <f>SUM(B21:E21)</f>
+        <f t="shared" si="5"/>
         <v>12311</v>
       </c>
       <c r="P21" s="6">
+        <f t="shared" si="6"/>
+        <v>14957</v>
+      </c>
+      <c r="Q21" s="6">
         <f t="shared" si="2"/>
-        <v>14957</v>
-      </c>
-      <c r="Q21" s="6">
-        <f t="shared" si="1"/>
         <v>17158.7</v>
       </c>
-      <c r="R21" s="12">
+      <c r="R21" s="10">
         <f>Q21*1.15</f>
         <v>19732.505000000001</v>
       </c>
-      <c r="S21" s="12">
+      <c r="S21" s="10">
         <f>R21*1.15</f>
         <v>22692.38075</v>
       </c>
-      <c r="T21" s="12">
+      <c r="T21" s="10">
         <f>S21*1.15</f>
         <v>26096.237862499998</v>
       </c>
-      <c r="U21" s="12">
-        <f t="shared" ref="U21:AH21" si="3">T21*1.03</f>
+      <c r="U21" s="10">
+        <f t="shared" ref="U21" si="10">T21*1.03</f>
         <v>26879.124998374999</v>
       </c>
-      <c r="V21" s="12">
-        <f>U21*1.15</f>
+      <c r="V21" s="10">
+        <f t="shared" ref="V21:AH21" si="11">U21*1.15</f>
         <v>30910.993748131245</v>
       </c>
-      <c r="W21" s="12">
-        <f>V21*1.15</f>
+      <c r="W21" s="10">
+        <f t="shared" si="11"/>
         <v>35547.642810350932</v>
       </c>
-      <c r="X21" s="12">
-        <f>W21*1.15</f>
+      <c r="X21" s="10">
+        <f t="shared" si="11"/>
         <v>40879.789231903567</v>
       </c>
-      <c r="Y21" s="12">
-        <f>X21*1.15</f>
+      <c r="Y21" s="10">
+        <f t="shared" si="11"/>
         <v>47011.757616689101</v>
       </c>
-      <c r="Z21" s="12">
-        <f>Y21*1.15</f>
+      <c r="Z21" s="10">
+        <f t="shared" si="11"/>
         <v>54063.521259192465</v>
       </c>
-      <c r="AA21" s="12">
-        <f>Z21*1.15</f>
+      <c r="AA21" s="10">
+        <f t="shared" si="11"/>
         <v>62173.049448071331</v>
       </c>
-      <c r="AB21" s="12">
-        <f>AA21*1.15</f>
+      <c r="AB21" s="10">
+        <f t="shared" si="11"/>
         <v>71499.006865282019</v>
       </c>
-      <c r="AC21" s="12">
-        <f>AB21*1.15</f>
+      <c r="AC21" s="10">
+        <f t="shared" si="11"/>
         <v>82223.85789507431</v>
       </c>
-      <c r="AD21" s="12">
-        <f>AC21*1.15</f>
+      <c r="AD21" s="10">
+        <f t="shared" si="11"/>
         <v>94557.436579335452</v>
       </c>
-      <c r="AE21" s="12">
-        <f>AD21*1.15</f>
+      <c r="AE21" s="10">
+        <f t="shared" si="11"/>
         <v>108741.05206623576</v>
       </c>
-      <c r="AF21" s="12">
-        <f>AE21*1.15</f>
+      <c r="AF21" s="10">
+        <f t="shared" si="11"/>
         <v>125052.20987617111</v>
       </c>
-      <c r="AG21" s="12">
-        <f>AF21*1.15</f>
+      <c r="AG21" s="10">
+        <f t="shared" si="11"/>
         <v>143810.04135759675</v>
       </c>
-      <c r="AH21" s="12">
-        <f>AG21*1.15</f>
+      <c r="AH21" s="10">
+        <f t="shared" si="11"/>
         <v>165381.54756123625</v>
       </c>
-      <c r="AI21" s="12"/>
+      <c r="AI21" s="10"/>
     </row>
     <row r="23" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="9">
-        <f xml:space="preserve"> B13/B2</f>
+      <c r="B23" s="8">
+        <f t="shared" ref="B23:M23" si="12" xml:space="preserve"> B13/B2</f>
         <v>0.6759275540706875</v>
       </c>
-      <c r="C23" s="9">
-        <f xml:space="preserve"> C13/C2</f>
+      <c r="C23" s="8">
+        <f t="shared" si="12"/>
         <v>0.62506545644964218</v>
       </c>
-      <c r="D23" s="9">
-        <f xml:space="preserve"> D13/D2</f>
+      <c r="D23" s="8">
+        <f t="shared" si="12"/>
         <v>0.66296900489396415</v>
       </c>
-      <c r="E23" s="9">
-        <f xml:space="preserve"> E13/E2</f>
+      <c r="E23" s="8">
+        <f t="shared" si="12"/>
         <v>0.65787467601768568</v>
       </c>
-      <c r="F23" s="9">
-        <f xml:space="preserve"> F13/F2</f>
+      <c r="F23" s="8">
+        <f t="shared" si="12"/>
         <v>0.67658308542286438</v>
       </c>
-      <c r="G23" s="9">
-        <f xml:space="preserve"> G13/G2</f>
+      <c r="G23" s="8">
+        <f t="shared" si="12"/>
         <v>0.66796494644595905</v>
       </c>
-      <c r="H23" s="9">
-        <f xml:space="preserve"> H13/H2</f>
+      <c r="H23" s="8">
+        <f t="shared" si="12"/>
         <v>0.57017182130584187</v>
       </c>
-      <c r="I23" s="9">
-        <f xml:space="preserve"> I13/I2</f>
+      <c r="I23" s="8">
+        <f t="shared" si="12"/>
         <v>0.6532682676255297</v>
       </c>
-      <c r="J23" s="9">
-        <f xml:space="preserve"> J13/J2</f>
+      <c r="J23" s="8">
+        <f t="shared" si="12"/>
         <v>0.64138104838709675</v>
       </c>
-      <c r="K23" s="9">
-        <f xml:space="preserve"> K13/K2</f>
+      <c r="K23" s="8">
+        <f t="shared" si="12"/>
         <v>0.66825297432686281</v>
       </c>
-      <c r="L23" s="9">
-        <f xml:space="preserve"> L13/L2</f>
+      <c r="L23" s="8">
+        <f t="shared" si="12"/>
         <v>0.6184907054044072</v>
       </c>
-      <c r="M23" s="9">
-        <f xml:space="preserve"> M13/M2</f>
+      <c r="M23" s="8">
+        <f t="shared" si="12"/>
         <v>0.64731428838273586</v>
       </c>
-      <c r="O23" s="9">
+      <c r="O23" s="8">
         <f xml:space="preserve"> O13/O2</f>
         <v>0.65563161169881767</v>
       </c>
-      <c r="P23" s="9">
+      <c r="P23" s="8">
         <f xml:space="preserve"> P13/P2</f>
         <v>0.64186284544524053</v>
       </c>
-      <c r="Q23" s="9">
+      <c r="Q23" s="8">
         <f xml:space="preserve"> Q13/Q2</f>
         <v>0.64381763708344453</v>
       </c>
@@ -2200,63 +2197,63 @@
       <c r="A24" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="10">
-        <f xml:space="preserve"> B21/B2</f>
+      <c r="B24" s="8">
+        <f t="shared" ref="B24:M24" si="13" xml:space="preserve"> B21/B2</f>
         <v>0.54967469667663094</v>
       </c>
-      <c r="C24" s="10">
-        <f xml:space="preserve"> C21/C2</f>
+      <c r="C24" s="8">
+        <f t="shared" si="13"/>
         <v>0.52818991097922852</v>
       </c>
-      <c r="D24" s="10">
-        <f xml:space="preserve"> D21/D2</f>
+      <c r="D24" s="8">
+        <f t="shared" si="13"/>
         <v>0.42006525285481239</v>
       </c>
-      <c r="E24" s="10">
-        <f xml:space="preserve"> E21/E2</f>
+      <c r="E24" s="8">
+        <f t="shared" si="13"/>
         <v>0.54642475987193173</v>
       </c>
-      <c r="F24" s="10">
-        <f xml:space="preserve"> F21/F2</f>
+      <c r="F24" s="8">
+        <f t="shared" si="13"/>
         <v>0.56084431222552766</v>
       </c>
-      <c r="G24" s="10">
-        <f xml:space="preserve"> G21/G2</f>
+      <c r="G24" s="8">
+        <f t="shared" si="13"/>
         <v>0.50730282375851998</v>
       </c>
-      <c r="H24" s="10">
-        <f xml:space="preserve"> H21/H2</f>
+      <c r="H24" s="8">
+        <f t="shared" si="13"/>
         <v>0.46886597938144331</v>
       </c>
-      <c r="I24" s="10">
-        <f xml:space="preserve"> I21/I2</f>
+      <c r="I24" s="8">
+        <f t="shared" si="13"/>
         <v>0.50597149094644922</v>
       </c>
-      <c r="J24" s="10">
-        <f xml:space="preserve"> J21/J2</f>
+      <c r="J24" s="8">
+        <f t="shared" si="13"/>
         <v>0.52658770161290325</v>
       </c>
-      <c r="K24" s="10">
-        <f xml:space="preserve"> K21/K2</f>
+      <c r="K24" s="8">
+        <f t="shared" si="13"/>
         <v>0.53312460864120226</v>
       </c>
-      <c r="L24" s="10">
-        <f xml:space="preserve"> L21/L2</f>
+      <c r="L24" s="8">
+        <f t="shared" si="13"/>
         <v>0.5116336328942509</v>
       </c>
-      <c r="M24" s="10">
-        <f xml:space="preserve"> M21/M2</f>
+      <c r="M24" s="8">
+        <f t="shared" si="13"/>
         <v>0.53313798055033457</v>
       </c>
-      <c r="O24" s="10">
+      <c r="O24" s="8">
         <f xml:space="preserve"> O21/O2</f>
         <v>0.51072391619995849</v>
       </c>
-      <c r="P24" s="10">
+      <c r="P24" s="8">
         <f xml:space="preserve"> P21/P2</f>
         <v>0.51030365063118388</v>
       </c>
-      <c r="Q24" s="10">
+      <c r="Q24" s="8">
         <f xml:space="preserve"> Q21/Q2</f>
         <v>0.52618392686838578</v>
       </c>
@@ -2265,59 +2262,59 @@
       <c r="A26" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="10" t="e">
+      <c r="B26" s="8" t="e">
         <f xml:space="preserve"> B2/#REF! -1</f>
         <v>#REF!</v>
       </c>
-      <c r="C26" s="10" t="e">
+      <c r="C26" s="8" t="e">
         <f xml:space="preserve"> C2/#REF! -1</f>
         <v>#REF!</v>
       </c>
-      <c r="D26" s="10" t="e">
+      <c r="D26" s="8" t="e">
         <f xml:space="preserve"> D2/#REF! -1</f>
         <v>#REF!</v>
       </c>
-      <c r="E26" s="10" t="e">
-        <f xml:space="preserve"> E2/A2 -1</f>
+      <c r="E26" s="8" t="e">
+        <f t="shared" ref="E26:M26" si="14" xml:space="preserve"> E2/A2 -1</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F26" s="10">
-        <f xml:space="preserve"> F2/B2 -1</f>
+      <c r="F26" s="8">
+        <f t="shared" si="14"/>
         <v>0.24125197819588529</v>
       </c>
-      <c r="G26" s="10">
-        <f xml:space="preserve"> G2/C2 -1</f>
+      <c r="G26" s="8">
+        <f t="shared" si="14"/>
         <v>0.25484377727352059</v>
       </c>
-      <c r="H26" s="10">
-        <f xml:space="preserve"> H2/D2 -1</f>
+      <c r="H26" s="8">
+        <f t="shared" si="14"/>
         <v>0.18678629690048942</v>
       </c>
-      <c r="I26" s="10">
-        <f xml:space="preserve"> I2/E2 -1</f>
+      <c r="I26" s="8">
+        <f t="shared" si="14"/>
         <v>0.18722366214361941</v>
       </c>
-      <c r="J26" s="10">
-        <f xml:space="preserve"> J2/F2 -1</f>
+      <c r="J26" s="8">
+        <f t="shared" si="14"/>
         <v>0.12423856070264905</v>
       </c>
-      <c r="K26" s="10">
-        <f xml:space="preserve"> K2/G2 -1</f>
+      <c r="K26" s="8">
+        <f t="shared" si="14"/>
         <v>0.11072471831965514</v>
       </c>
-      <c r="L26" s="10">
-        <f xml:space="preserve"> L2/H2 -1</f>
+      <c r="L26" s="8">
+        <f t="shared" si="14"/>
         <v>0.11656357388316141</v>
       </c>
-      <c r="M26" s="10">
-        <f xml:space="preserve"> M2/I2 -1</f>
+      <c r="M26" s="8">
+        <f t="shared" si="14"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="P26" s="10">
+      <c r="P26" s="8">
         <f>P2/O2 - 1</f>
         <v>0.21593030491599263</v>
       </c>
-      <c r="Q26" s="10">
+      <c r="Q26" s="8">
         <f>Q2/P2 - 1</f>
         <v>0.11257932446264074</v>
       </c>
@@ -2326,59 +2323,59 @@
       <c r="A27" t="s">
         <v>46</v>
       </c>
-      <c r="B27" s="10" t="e">
+      <c r="B27" s="8" t="e">
         <f xml:space="preserve"> B21/#REF! - 1</f>
         <v>#REF!</v>
       </c>
-      <c r="C27" s="10" t="e">
+      <c r="C27" s="8" t="e">
         <f xml:space="preserve"> C21/#REF! - 1</f>
         <v>#REF!</v>
       </c>
-      <c r="D27" s="10" t="e">
+      <c r="D27" s="8" t="e">
         <f xml:space="preserve"> D21/#REF! - 1</f>
         <v>#REF!</v>
       </c>
-      <c r="E27" s="10" t="e">
-        <f xml:space="preserve"> E21/A21 - 1</f>
+      <c r="E27" s="8" t="e">
+        <f t="shared" ref="E27:M27" si="15" xml:space="preserve"> E21/A21 - 1</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F27" s="10">
-        <f xml:space="preserve"> F21/B21 - 1</f>
+      <c r="F27" s="8">
+        <f t="shared" si="15"/>
         <v>0.26647472808701211</v>
       </c>
-      <c r="G27" s="10">
-        <f xml:space="preserve"> G21/C21 - 1</f>
+      <c r="G27" s="8">
+        <f t="shared" si="15"/>
         <v>0.20522141440846009</v>
       </c>
-      <c r="H27" s="10">
-        <f xml:space="preserve"> H21/D21 - 1</f>
+      <c r="H27" s="8">
+        <f t="shared" si="15"/>
         <v>0.32466019417475733</v>
       </c>
-      <c r="I27" s="10">
-        <f xml:space="preserve"> I21/E21 - 1</f>
+      <c r="I27" s="8">
+        <f t="shared" si="15"/>
         <v>9.9330357142857206E-2</v>
       </c>
-      <c r="J27" s="10">
-        <f xml:space="preserve"> J21/F21 - 1</f>
+      <c r="J27" s="8">
+        <f t="shared" si="15"/>
         <v>5.5569588279868576E-2</v>
       </c>
-      <c r="K27" s="10">
-        <f xml:space="preserve"> K21/G21 - 1</f>
+      <c r="K27" s="8">
+        <f t="shared" si="15"/>
         <v>0.16726076227035924</v>
       </c>
-      <c r="L27" s="10">
-        <f xml:space="preserve"> L21/H21 - 1</f>
+      <c r="L27" s="8">
+        <f t="shared" si="15"/>
         <v>0.21841102316036354</v>
       </c>
-      <c r="M27" s="10">
-        <f xml:space="preserve"> M21/I21 - 1</f>
+      <c r="M27" s="8">
+        <f t="shared" si="15"/>
         <v>0.15906091370558384</v>
       </c>
-      <c r="P27" s="10">
+      <c r="P27" s="8">
         <f xml:space="preserve"> P21/O21 - 1</f>
         <v>0.21492973763301104</v>
       </c>
-      <c r="Q27" s="10">
+      <c r="Q27" s="8">
         <f xml:space="preserve"> Q21/P21 - 1</f>
         <v>0.14720197900648535</v>
       </c>
@@ -2420,7 +2417,7 @@
       <c r="R31" t="s">
         <v>126</v>
       </c>
-      <c r="S31" s="10">
+      <c r="S31" s="8">
         <v>0.08</v>
       </c>
     </row>
@@ -2441,7 +2438,7 @@
       <c r="R32" t="s">
         <v>127</v>
       </c>
-      <c r="S32" s="14">
+      <c r="S32" s="11">
         <f>NPV(S31,Q21:AH21)</f>
         <v>467680.55903581879</v>
       </c>
@@ -3047,7 +3044,7 @@
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A84" s="8" t="s">
+      <c r="A84" t="s">
         <v>90</v>
       </c>
     </row>
@@ -3060,7 +3057,7 @@
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A86" s="8" t="s">
+      <c r="A86" t="s">
         <v>91</v>
       </c>
       <c r="B86" s="3">
@@ -3076,7 +3073,7 @@
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A88" s="8" t="s">
+      <c r="A88" t="s">
         <v>93</v>
       </c>
       <c r="B88" s="3">
@@ -3092,7 +3089,7 @@
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A90" s="8" t="s">
+      <c r="A90" t="s">
         <v>95</v>
       </c>
       <c r="B90" s="3">
@@ -3203,7 +3200,7 @@
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A106" s="8" t="s">
+      <c r="A106" t="s">
         <v>76</v>
       </c>
       <c r="B106" s="3"/>
@@ -3217,7 +3214,7 @@
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A108" s="8" t="s">
+      <c r="A108" t="s">
         <v>107</v>
       </c>
       <c r="B108" s="3">
@@ -3233,7 +3230,7 @@
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A110" s="8" t="s">
+      <c r="A110" t="s">
         <v>112</v>
       </c>
       <c r="B110" s="3">
@@ -3249,7 +3246,7 @@
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A112" s="8" t="s">
+      <c r="A112" t="s">
         <v>110</v>
       </c>
       <c r="B112" s="3">
@@ -3753,7 +3750,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="8" t="s">
+      <c r="A23" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3763,7 +3760,7 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="8" t="s">
+      <c r="A25" t="s">
         <v>151</v>
       </c>
     </row>
@@ -3802,7 +3799,7 @@
       <c r="B36" s="3">
         <v>3668</v>
       </c>
-      <c r="C36" s="10">
+      <c r="C36" s="8">
         <f>B36/B41</f>
         <v>0.45155730641388647</v>
       </c>
@@ -3814,7 +3811,7 @@
       <c r="B37" s="3">
         <v>4105</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="8">
         <f xml:space="preserve"> B37/B41</f>
         <v>0.5053551643481472</v>
       </c>
@@ -3826,7 +3823,7 @@
       <c r="B38" s="3">
         <v>2920</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="8">
         <f xml:space="preserve"> B38/B41</f>
         <v>0.35947310107103286</v>
       </c>

</xml_diff>